<commit_message>
feat(mqtt): Sprint 1 Backend concluido — MQTT listener + historico paginado
- DiagnosticoEvento model: device_id, classe, confianca, temp, umidade, timestamp
- mqtt_listener: retry exponencial, shutdown SIGTERM/SIGINT limpo
- GET /api/diagnostico/historico/ paginado page_size=10
- Mosquitto 2.1.2 instalado e configurado (localhost:1883)
- 5/5 testes passando
</commit_message>
<xml_diff>
--- a/docs/Backlog_Ceres_Diagnostico_v2_atualizado.xlsx
+++ b/docs/Backlog_Ceres_Diagnostico_v2_atualizado.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produto" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escrita TCC e Artigo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Produto" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Escrita TCC e Artigo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -115,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -137,11 +137,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -209,6 +253,8 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -574,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -590,7 +636,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backlog do Produto — Ceres Diagnóstico v2  |  IFMT Sorriso-MT  |  Namem Rachid Jaudy Neto</t>
+          <t>Backlog do Produto — Ceres Diagnóstico v2  |  IFMT Cuiaba  |  Namem Rachid Jaudy Neto</t>
         </is>
       </c>
     </row>
@@ -948,11 +994,42 @@
       <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Sprint 1 — MQTT + Dataset + Treino 🔄 EM ANDAMENTO</t>
-        </is>
-      </c>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Criar firmware/esp32_mqtt_sensor/ com PlatformIO (esp32dev)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>🔄 Em andamento</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>ESP32</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Projeto compila sem erro</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -967,7 +1044,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Criar firmware/esp32_mqtt_sensor/ com PlatformIO (esp32dev)</t>
+          <t>DHT22 GPIO4 + sensor solo GPIO34 + publicação MQTT a cada 30s</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -987,7 +1064,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Projeto compila sem erro</t>
+          <t>JSON publicado em ceres/sensor/001</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
@@ -1005,12 +1082,12 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>DHT22 GPIO4 + sensor solo GPIO34 + publicação MQTT a cada 30s</t>
+          <t>Reconexão automática WiFi e MQTT</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1025,7 +1102,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>JSON publicado em ceres/sensor/001</t>
+          <t>Reconecta após queda sem reiniciar</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
@@ -1038,17 +1115,17 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Reconexão automática WiFi e MQTT</t>
+          <t>Adicionar paho-mqtt&gt;=2.0.0 ao requirements.txt</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1058,12 +1135,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>ESP32</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Reconecta após queda sem reiniciar</t>
+          <t>pip install sem erros</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>
@@ -1081,7 +1158,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Adicionar paho-mqtt&gt;=2.0.0 ao requirements.txt</t>
+          <t>Model DiagnosticoEvento + migration</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1101,7 +1178,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>pip install sem erros</t>
+          <t>Evento salvo no banco ao receber MQTT</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr"/>
@@ -1119,7 +1196,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Model DiagnosticoEvento + migration</t>
+          <t>Command mqtt_listener (retry exponencial + shutdown SIGTERM)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1139,7 +1216,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Evento salvo no banco ao receber MQTT</t>
+          <t>Subscreve ceres/sensor/# e persiste eventos</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr"/>
@@ -1157,7 +1234,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Command mqtt_listener (retry exponencial + shutdown SIGTERM)</t>
+          <t>Endpoint GET /api/diagnostico/historico/ paginado (page_size=10)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1177,7 +1254,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Subscreve ceres/sensor/# e persiste eventos</t>
+          <t>Últimos 20 eventos retornados</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr"/>
@@ -1195,12 +1272,12 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Endpoint GET /api/diagnostico/historico/ paginado (page_size=10)</t>
+          <t>Testes: evento_criado_com_dados_validos e historico_paginado</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1215,7 +1292,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Últimos 20 eventos retornados</t>
+          <t>python manage.py test passa</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr"/>
@@ -1228,35 +1305,39 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Dataset</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Testes: evento_criado_com_dados_validos e historico_paginado</t>
+          <t>Baixar PlantVillage do Kaggle (abdallahalidev/plantvillage-dataset)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Crítica</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>🔄 Em andamento</t>
+          <t>✅ Concluído</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>python manage.py test passa</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr"/>
+          <t>~18.160 imagens disponíveis localmente</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>18.160 imgs, 10 classes tomate — 2026-04-28</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -1271,17 +1352,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Baixar PlantVillage do Kaggle (abdallahalidev/plantvillage-dataset)</t>
+          <t>Script prepare_plantvillage.py (10 classes, split 70/15/15, augmentation)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Crítica</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>🔄 Em andamento</t>
+          <t>✅ Concluído</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1291,12 +1372,12 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>~18.160 imagens disponíveis localmente</t>
+          <t>Estrutura train/val/test gerada, mín 500 imgs/classe</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>NÃO usar Roboflow Fruit</t>
+          <t>88.949 imgs treino (augm. offline x6), split 70/15/15, seed=42</t>
         </is>
       </c>
     </row>
@@ -1313,17 +1394,17 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Script prepare_plantvillage.py (10 classes, split 70/15/15, augmentation)</t>
+          <t>Gerar dataset_stats.md + edge_impulse_upload_guide.md</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>🔄 Em andamento</t>
+          <t>✅ Concluído</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1333,10 +1414,14 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Estrutura train/val/test gerada, mín 500 imgs/classe</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr"/>
+          <t>Documentação do dataset gerada</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Gerados em 2026-04-28</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
@@ -1346,22 +1431,22 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Dataset</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Gerar dataset_stats.md + edge_impulse_upload_guide.md</t>
+          <t>Treinar MobileNetV2 INT8 — Exp A (Edge Impulse) e Exp B (TF local WSL2)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>🔄 Em andamento</t>
+          <t>✅ Concluído</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1371,53 +1456,61 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Documentação do dataset gerada</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr"/>
+          <t>Modelo treinado e pronto para exportação</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Exp A: FP32 92.5%/INT8 62.0% val acc (EI, quantizacao automatica sem calibracao) | Exp B: INT8 98.13% test acc 639KB (TF local, 2 fases, calibracao real) &lt;- ESCOLHIDO Sprint 2</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Treinar MobileNetV2 INT8 no Edge Impulse</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 2 — ESP32-S3 + TFLite + Integração Completa ⏳ PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>PlatformIO ESP32-S3 N16R8 (Flash 16MB, PSRAM habilitada)</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>🔄 Em andamento</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Modelo treinado e pronto para exportação</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 2 — ESP32-S3 + TFLite + Integração Completa ⏳ PENDENTE</t>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>⏳ Pendente</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>ESP32-S3</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Projeto compila e roda na placa</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Aguardando chegada da placa</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1527,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>PlatformIO ESP32-S3 N16R8 (Flash 16MB, PSRAM habilitada)</t>
+          <t>Sketch teste câmera OV5640 com pinout correto para N16R8</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1454,14 +1547,10 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Projeto compila e roda na placa</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Aguardando chegada da placa</t>
-        </is>
-      </c>
+          <t>Frame capturado e tamanho impresso no serial</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -1476,12 +1565,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Sketch teste câmera OV5640 com pinout correto para N16R8</t>
+          <t>Documentar gravação via USB-C nativo (sem FTDI)</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baixa</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1496,7 +1585,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Frame capturado e tamanho impresso no serial</t>
+          <t>README com passos de gravação</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -1509,17 +1598,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>TFLite</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Documentar gravação via USB-C nativo (sem FTDI)</t>
+          <t>Exportar modelo do Edge Impulse como Arduino Library</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Baixa</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1529,12 +1618,12 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>ESP32-S3</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>README com passos de gravação</t>
+          <t>Modelo exportado após treino da Sprint 1</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr"/>
@@ -1552,7 +1641,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Exportar modelo do Edge Impulse como Arduino Library</t>
+          <t>Integrar biblioteca ao PlatformIO (lib/ei_ceres/)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1567,12 +1656,12 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>ESP32-S3</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Modelo exportado após treino da Sprint 1</t>
+          <t>Compila com modelo integrado</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -1590,7 +1679,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Integrar biblioteca ao PlatformIO (lib/ei_ceres/)</t>
+          <t>inference.h/cpp: alocação PSRAM, normalização, latência esp_timer</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1610,7 +1699,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Compila com modelo integrado</t>
+          <t>Latência &lt; 300ms, RAM livre &gt; 4MB</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr"/>
@@ -1623,12 +1712,12 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>TFLite</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>inference.h/cpp: alocação PSRAM, normalização, latência esp_timer</t>
+          <t>Ciclo completo: OV5640 → inferência → DHT22 + solo → MQTT</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1648,7 +1737,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Latência &lt; 300ms, RAM livre &gt; 4MB</t>
+          <t>Threshold 0.70, JSON publicado</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -1666,12 +1755,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Ciclo completo: OV5640 → inferência → DHT22 + solo → MQTT</t>
+          <t>LED indicadores + NVS + Watchdog 60s + reconexão automática</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
@@ -1686,7 +1775,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Threshold 0.70, JSON publicado</t>
+          <t>Firmware robusto sem supervisão humana</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr"/>
@@ -1699,17 +1788,17 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Benchmark</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>LED indicadores + NVS + Watchdog 60s + reconexão automática</t>
+          <t>Script benchmark_esp32s3.py (50 imgs, latência + acurácia)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -1719,12 +1808,12 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>ESP32-S3</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Firmware robusto sem supervisão humana</t>
+          <t>Latência média/p95, acurácia por classe gerados</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -1742,7 +1831,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Script benchmark_esp32s3.py (50 imgs, latência + acurácia)</t>
+          <t>Gerar benchmark_results.md + benchmark_raw.csv</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -1762,7 +1851,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Latência média/p95, acurácia por classe gerados</t>
+          <t>Dados prontos para o artigo (Capítulo 4)</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr"/>
@@ -1780,12 +1869,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Gerar benchmark_results.md + benchmark_raw.csv</t>
+          <t>Comparativo edge vs Python local com tflite-runtime</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -1800,7 +1889,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Dados prontos para o artigo (Capítulo 4)</t>
+          <t>Tabela comparativa gerada</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -1813,17 +1902,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Benchmark</t>
+          <t>Integração</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Comparativo edge vs Python local com tflite-runtime</t>
+          <t>Teste end-to-end: T0→T4 para 5 eventos, meta &lt; 5s</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -1833,12 +1922,12 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Tabela comparativa gerada</t>
+          <t>Tempo total medido e documentado</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr"/>
@@ -1849,82 +1938,58 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Integração</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Teste end-to-end: T0→T4 para 5 eventos, meta &lt; 5s</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="B37" s="23" t="n"/>
+      <c r="C37" s="23" t="n"/>
+      <c r="D37" s="23" t="n"/>
+      <c r="E37" s="23" t="n"/>
+      <c r="F37" s="23" t="n"/>
+      <c r="G37" s="23" t="n"/>
+      <c r="H37" s="24" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 3 — Flutter + Resiliência + Experimentos ⏳ PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Flutter</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Design System Agrícola (Mobile First) — ícones, fotos, mín. digitação</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>⏳ Pendente</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>Full Stack</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Tempo total medido e documentado</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Integração</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Documentar e2e_test_results.md com tabela T0→T4</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>⏳ Pendente</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>Full Stack</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>Gargalos identificados e corrigidos</t>
-        </is>
-      </c>
-      <c r="H38" s="5" t="inlineStr"/>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 3 — Flutter + Resiliência + Experimentos ⏳ PENDENTE</t>
-        </is>
-      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>⏳ Pendente</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Interface validada para uso em campo</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
@@ -1939,7 +2004,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Design System Agrícola (Mobile First) — ícones, fotos, mín. digitação</t>
+          <t>DiagnosticoResultadoScreen (nome, confiança, sensores, recomendação)</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -1959,7 +2024,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Interface validada para uso em campo</t>
+          <t>Exibe resultado completo da inferência</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr"/>
@@ -1977,7 +2042,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>DiagnosticoResultadoScreen (nome, confiança, sensores, recomendação)</t>
+          <t>HistoricoScreen com paginação infinita e pull-to-refresh</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -1997,7 +2062,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Exibe resultado completo da inferência</t>
+          <t>Consome GET /api/diagnostico/historico/</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -2015,12 +2080,12 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>HistoricoScreen com paginação infinita e pull-to-refresh</t>
+          <t>SensorStatusScreen com polling a cada 10s (online/offline)</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
@@ -2035,7 +2100,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Consome GET /api/diagnostico/historico/</t>
+          <t>Status do sensor exibido em tempo real</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr"/>
@@ -2053,7 +2118,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>SensorStatusScreen com polling a cada 10s (online/offline)</t>
+          <t>Integração com câmera para registro de foto da planta</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -2073,7 +2138,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Status do sensor exibido em tempo real</t>
+          <t>Foto anexada à triagem</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -2091,12 +2156,12 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Integração com câmera para registro de foto da planta</t>
+          <t>DiagnosticoEventoModel + DiagnosticoService em Dart</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -2111,7 +2176,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Foto anexada à triagem</t>
+          <t>flutter analyze sem warnings críticos</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr"/>
@@ -2124,12 +2189,12 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Flutter</t>
+          <t>Resiliência</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>DiagnosticoEventoModel + DiagnosticoService em Dart</t>
+          <t>Persistência offline com Drift (diagnóstico sem internet)</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -2149,7 +2214,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>flutter analyze sem warnings críticos</t>
+          <t>App funciona na lavoura sem conexão</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -2167,7 +2232,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Persistência offline com Drift (diagnóstico sem internet)</t>
+          <t>Módulo de sincronização inteligente (upload ao reconectar)</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -2182,12 +2247,12 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>App</t>
+          <t>App/Backend</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>App funciona na lavoura sem conexão</t>
+          <t>Dados enviados sem perda ao reconectar</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr"/>
@@ -2200,17 +2265,17 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>Resiliência</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Módulo de sincronização inteligente (upload ao reconectar)</t>
+          <t>Histórico de diagnósticos georreferenciados</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -2220,12 +2285,12 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>App/Backend</t>
+          <t>App</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Dados enviados sem perda ao reconectar</t>
+          <t>Mapa simples + lista de triagens anteriores</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -2243,12 +2308,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Histórico de diagnósticos georreferenciados</t>
+          <t>Módulo de recomendação de manejo automático pós-diagnóstico</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -2258,12 +2323,12 @@
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>App</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Mapa simples + lista de triagens anteriores</t>
+          <t>Orientações técnicas geradas automaticamente</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr"/>
@@ -2281,12 +2346,12 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Módulo de recomendação de manejo automático pós-diagnóstico</t>
+          <t>Sistema multi-tenant para associações/cooperativas</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -2301,7 +2366,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Orientações técnicas geradas automaticamente</t>
+          <t>Dados isolados por tenant</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -2314,12 +2379,12 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Gestão</t>
+          <t>Infraestrutura</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Sistema multi-tenant para associações/cooperativas</t>
+          <t>CI/CD e monitoramento configurados</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -2334,12 +2399,12 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Dados isolados por tenant</t>
+          <t>Pipeline de deploy automatizado</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr"/>
@@ -2357,12 +2422,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>CI/CD e monitoramento configurados</t>
+          <t>Relatórios técnicos (PDF/CSV) para agrônomos</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Baixa</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -2372,12 +2437,12 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Pipeline de deploy automatizado</t>
+          <t>Exportação disponível no painel</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -2390,17 +2455,17 @@
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>Infraestrutura</t>
+          <t>Experimento</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Relatórios técnicos (PDF/CSV) para agrônomos</t>
+          <t>Script experiment_edge_vs_cloud.py (100 imgs, +200ms overhead 4G)</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Baixa</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
@@ -2410,12 +2475,12 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>Exportação disponível no painel</t>
+          <t>Latência, acurácia e consumo comparados</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr"/>
@@ -2433,7 +2498,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Script experiment_edge_vs_cloud.py (100 imgs, +200ms overhead 4G)</t>
+          <t>Gerar experiment_a_results.md (tabela + gráfico ASCII)</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
@@ -2453,49 +2518,12 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Latência, acurácia e consumo comparados</t>
+          <t>Dados prontos para o artigo (Capítulo 5)</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
     </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="12" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>Experimento</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Gerar experiment_a_results.md (tabela + gráfico ASCII)</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>⏳ Pendente</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>Dados prontos para o artigo (Capítulo 5)</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr"/>
-    </row>
+    <row r="54" ht="30" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A12:H12"/>
@@ -2945,7 +2973,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Apresentação para banca — IFMT Sorriso-MT</t>
+          <t>Apresentação para banca — IFMT Cuiaba</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -3090,10 +3118,10 @@
         </is>
       </c>
       <c r="D4" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">

</xml_diff>